<commit_message>
Updated Counterfactual testing data
</commit_message>
<xml_diff>
--- a/data/ARID_DrugMoleculeTesting_CounterfactualTesting.xlsx
+++ b/data/ARID_DrugMoleculeTesting_CounterfactualTesting.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowHeight="17640"/>
+    <workbookView windowWidth="27900" windowHeight="11760"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="174" uniqueCount="53">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="173" uniqueCount="54">
   <si>
     <t>Acid (name)</t>
   </si>
@@ -71,109 +71,112 @@
     <t>Reaction_Yield</t>
   </si>
   <si>
+    <t>DeCIPHER_Predicted_Yield</t>
+  </si>
+  <si>
+    <t>References</t>
+  </si>
+  <si>
+    <t>4-chlorobenzoic acid</t>
+  </si>
+  <si>
+    <t>O=C(O)C1=CC=C(Cl)C=C1</t>
+  </si>
+  <si>
+    <t>2-morpholinoethan-1-amine</t>
+  </si>
+  <si>
+    <t>NCCN1CCOCC1</t>
+  </si>
+  <si>
+    <t>EDC.HCl</t>
+  </si>
+  <si>
+    <t>CN(C)CCCN=C=NCC.Cl</t>
+  </si>
+  <si>
+    <t>Pyridine</t>
+  </si>
+  <si>
+    <t>C1=NC=CC=C1</t>
+  </si>
+  <si>
+    <t>PS-750-M</t>
+  </si>
+  <si>
+    <t>O=C(OCCOCCOCCOCCOCCOCCOCCOCCOCCOCCOCCOCCOCCOCCOCCOCCOC)C1N(C(CCCCCCCCCCCC)=O)CCC1</t>
+  </si>
+  <si>
+    <t>https://pubs.acs.org/doi/10.1021/acs.orglett.0c01676.</t>
+  </si>
+  <si>
+    <t>2-(methylamino)-3,3-diphenylpropanoic acid</t>
+  </si>
+  <si>
+    <t>O=C(O)C(NC)C(C1=CC=CC=C1)C2=CC=CC=C2</t>
+  </si>
+  <si>
+    <t>4-fluoropyrrolidine-2-carboxamide</t>
+  </si>
+  <si>
+    <t>O=C(C1NCC(F)C1)N</t>
+  </si>
+  <si>
+    <t>3,4,5-trimethoxybenzoic acid</t>
+  </si>
+  <si>
+    <t>O=C(O)C1=CC(OC)=C(OC)C(OC)=C1</t>
+  </si>
+  <si>
+    <t>2-(4-(aminomethyl)phenoxy)-N,N-dimethylethan-1-amine</t>
+  </si>
+  <si>
+    <t>CN(C)CCOC1=CC=C(CN)C=C1</t>
+  </si>
+  <si>
+    <t>acetic acid</t>
+  </si>
+  <si>
+    <t>CC(O)=O</t>
+  </si>
+  <si>
+    <t>4-aminophenol</t>
+  </si>
+  <si>
+    <t>OC1=CC=C(N)C=C1</t>
+  </si>
+  <si>
+    <t>2-(4-hydroxyphenyl)acetic acid</t>
+  </si>
+  <si>
+    <t>O=C(O)CC1=CC=C(O)C=C1</t>
+  </si>
+  <si>
+    <t>3,5-dimethylaniline</t>
+  </si>
+  <si>
+    <t>NC1=CC(C)=CC(C)=C1</t>
+  </si>
+  <si>
+    <t>4-aminobenzoic acid</t>
+  </si>
+  <si>
+    <t>O=C(O)C1=CC=C(N)C=C1</t>
+  </si>
+  <si>
+    <t>2,6-dimethylaniline</t>
+  </si>
+  <si>
+    <t>NC1=C(C)C=CC=C1C</t>
+  </si>
+  <si>
+    <t>Experimental_Yield</t>
+  </si>
+  <si>
     <t>Predicted_Yield_Before</t>
   </si>
   <si>
     <t>Predicted_Yield_July4</t>
-  </si>
-  <si>
-    <t>References</t>
-  </si>
-  <si>
-    <t>4-chlorobenzoic acid</t>
-  </si>
-  <si>
-    <t>O=C(O)C1=CC=C(Cl)C=C1</t>
-  </si>
-  <si>
-    <t>2-morpholinoethan-1-amine</t>
-  </si>
-  <si>
-    <t>NCCN1CCOCC1</t>
-  </si>
-  <si>
-    <t>EDC.HCl</t>
-  </si>
-  <si>
-    <t>CN(C)CCCN=C=NCC.Cl</t>
-  </si>
-  <si>
-    <t>Pyridine</t>
-  </si>
-  <si>
-    <t>C1=NC=CC=C1</t>
-  </si>
-  <si>
-    <t>PS-750-M</t>
-  </si>
-  <si>
-    <t>O=C(OCCOCCOCCOCCOCCOCCOCCOCCOCCOCCOCCOCCOCCOCCOCCOCCOC)C1N(C(CCCCCCCCCCCC)=O)CCC1</t>
-  </si>
-  <si>
-    <t>https://pubs.acs.org/doi/10.1021/acs.orglett.0c01676.</t>
-  </si>
-  <si>
-    <t>2-(methylamino)-3,3-diphenylpropanoic acid</t>
-  </si>
-  <si>
-    <t>O=C(O)C(NC)C(C1=CC=CC=C1)C2=CC=CC=C2</t>
-  </si>
-  <si>
-    <t>4-fluoropyrrolidine-2-carboxamide</t>
-  </si>
-  <si>
-    <t>O=C(C1NCC(F)C1)N</t>
-  </si>
-  <si>
-    <t>3,4,5-trimethoxybenzoic acid</t>
-  </si>
-  <si>
-    <t>O=C(O)C1=CC(OC)=C(OC)C(OC)=C1</t>
-  </si>
-  <si>
-    <t>2-(4-(aminomethyl)phenoxy)-N,N-dimethylethan-1-amine</t>
-  </si>
-  <si>
-    <t>CN(C)CCOC1=CC=C(CN)C=C1</t>
-  </si>
-  <si>
-    <t>acetic acid</t>
-  </si>
-  <si>
-    <t>CC(O)=O</t>
-  </si>
-  <si>
-    <t>4-aminophenol</t>
-  </si>
-  <si>
-    <t>OC1=CC=C(N)C=C1</t>
-  </si>
-  <si>
-    <t>2-(4-hydroxyphenyl)acetic acid</t>
-  </si>
-  <si>
-    <t>O=C(O)CC1=CC=C(O)C=C1</t>
-  </si>
-  <si>
-    <t>3,5-dimethylaniline</t>
-  </si>
-  <si>
-    <t>NC1=CC(C)=CC(C)=C1</t>
-  </si>
-  <si>
-    <t>4-aminobenzoic acid</t>
-  </si>
-  <si>
-    <t>O=C(O)C1=CC=C(N)C=C1</t>
-  </si>
-  <si>
-    <t>2,6-dimethylaniline</t>
-  </si>
-  <si>
-    <t>NC1=C(C)C=CC=C1C</t>
-  </si>
-  <si>
-    <t>Experimental_Yield</t>
   </si>
 </sst>
 </file>
@@ -181,9 +184,9 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="4">
-    <numFmt numFmtId="42" formatCode="_(&quot;$&quot;* #,##0_);_(&quot;$&quot;* \(#,##0\);_(&quot;$&quot;* &quot;-&quot;_);_(@_)"/>
     <numFmt numFmtId="176" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
     <numFmt numFmtId="177" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
+    <numFmt numFmtId="42" formatCode="_(&quot;$&quot;* #,##0_);_(&quot;$&quot;* \(#,##0\);_(&quot;$&quot;* &quot;-&quot;_);_(@_)"/>
     <numFmt numFmtId="44" formatCode="_(&quot;$&quot;* #,##0.00_);_(&quot;$&quot;* \(#,##0.00\);_(&quot;$&quot;* &quot;-&quot;??_);_(@_)"/>
   </numFmts>
   <fonts count="24">
@@ -216,6 +219,97 @@
       <color rgb="FF00B050"/>
       <name val="Arial"/>
       <charset val="134"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="13"/>
+      <color theme="3"/>
+      <name val="Calibri"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF9C6500"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color rgb="FF800080"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FFFF0000"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="18"/>
+      <color theme="3"/>
+      <name val="Calibri"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="0"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="15"/>
+      <color theme="3"/>
+      <name val="Calibri"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <i/>
+      <sz val="11"/>
+      <color rgb="FF7F7F7F"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="3"/>
+      <name val="Calibri"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF3F3F76"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FFFA7D00"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
     </font>
     <font>
       <u/>
@@ -228,32 +322,9 @@
     <font>
       <b/>
       <sz val="11"/>
-      <color rgb="FFFFFFFF"/>
+      <color rgb="FF3F3F3F"/>
       <name val="Calibri"/>
       <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color theme="0"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <u/>
-      <sz val="11"/>
-      <color rgb="FF800080"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color theme="3"/>
-      <name val="Calibri"/>
-      <charset val="134"/>
       <scheme val="minor"/>
     </font>
     <font>
@@ -264,39 +335,16 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <b/>
       <sz val="11"/>
-      <color rgb="FFFA7D00"/>
+      <color rgb="FF9C0006"/>
       <name val="Calibri"/>
       <charset val="0"/>
       <scheme val="minor"/>
     </font>
     <font>
       <b/>
-      <sz val="15"/>
-      <color theme="3"/>
-      <name val="Calibri"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
       <sz val="11"/>
-      <color rgb="FF3F3F3F"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF3F3F76"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color theme="1"/>
+      <color rgb="FFFFFFFF"/>
       <name val="Calibri"/>
       <charset val="0"/>
       <scheme val="minor"/>
@@ -310,57 +358,12 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <b/>
-      <sz val="13"/>
-      <color theme="3"/>
-      <name val="Calibri"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF9C0006"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
       <sz val="11"/>
       <color rgb="FFFA7D00"/>
       <name val="Calibri"/>
       <charset val="0"/>
       <scheme val="minor"/>
     </font>
-    <font>
-      <b/>
-      <sz val="18"/>
-      <color theme="3"/>
-      <name val="Calibri"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF9C6500"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <i/>
-      <sz val="11"/>
-      <color rgb="FF7F7F7F"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FFFF0000"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
   </fonts>
   <fills count="35">
     <fill>
@@ -383,91 +386,145 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor rgb="FFFFEB9C"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFCC99"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFFCC"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFF2F2F2"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFC6EFCE"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFC7CE"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor rgb="FFA5A5A5"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFC6EFCE"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFF2F2F2"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFFFCC"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFCC99"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
         <fgColor theme="9" tint="0.599993896298105"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFFFC7CE"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.799981688894314"/>
+        <fgColor theme="7" tint="0.599993896298105"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -479,7 +536,25 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.799981688894314"/>
+        <fgColor theme="5"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.399975585192419"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -491,79 +566,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
         <fgColor theme="8" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFEB9C"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.599993896298105"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -610,26 +613,11 @@
       <diagonal/>
     </border>
     <border>
-      <left style="double">
-        <color rgb="FF3F3F3F"/>
-      </left>
-      <right style="double">
-        <color rgb="FF3F3F3F"/>
-      </right>
-      <top style="double">
-        <color rgb="FF3F3F3F"/>
-      </top>
-      <bottom style="double">
-        <color rgb="FF3F3F3F"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
       <left/>
       <right/>
       <top/>
       <bottom style="medium">
-        <color theme="4" tint="0.499984740745262"/>
+        <color theme="4"/>
       </bottom>
       <diagonal/>
     </border>
@@ -645,15 +633,6 @@
       </top>
       <bottom style="thin">
         <color rgb="FF7F7F7F"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="medium">
-        <color theme="4"/>
       </bottom>
       <diagonal/>
     </border>
@@ -690,6 +669,30 @@
     <border>
       <left/>
       <right/>
+      <top/>
+      <bottom style="medium">
+        <color theme="4" tint="0.499984740745262"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="double">
+        <color rgb="FF3F3F3F"/>
+      </left>
+      <right style="double">
+        <color rgb="FF3F3F3F"/>
+      </right>
+      <top style="double">
+        <color rgb="FF3F3F3F"/>
+      </top>
+      <bottom style="double">
+        <color rgb="FF3F3F3F"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
       <top style="thin">
         <color theme="4"/>
       </top>
@@ -710,152 +713,152 @@
   </borders>
   <cellStyleXfs count="49">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="7" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="11" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="10" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="7" borderId="9" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="11" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="11" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="10" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="12" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="44" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="8" borderId="8" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="9" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="10" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="6" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="9" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="12" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="4" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="176" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="5" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="7" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="5" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="7" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="176" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="42" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="7" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="4" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="177" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="4" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="5" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="21" fillId="25" borderId="9" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="9" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
@@ -885,9 +888,6 @@
       <alignment horizontal="left" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1239,7 +1239,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:U7"/>
+  <dimension ref="A1:T7"/>
   <sheetFormatPr defaultColWidth="8.8359375" defaultRowHeight="18.4" outlineLevelRow="6"/>
   <cols>
     <col min="1" max="1" width="56" style="3" customWidth="1"/>
@@ -1260,13 +1260,12 @@
     <col min="16" max="16" width="13.1640625" style="3" customWidth="1"/>
     <col min="17" max="17" width="12" style="3" customWidth="1"/>
     <col min="18" max="18" width="27" style="3" customWidth="1"/>
-    <col min="19" max="19" width="32.6640625" style="3" customWidth="1"/>
-    <col min="20" max="20" width="31" style="3" customWidth="1"/>
-    <col min="21" max="21" width="67.3359375" style="10" customWidth="1"/>
-    <col min="22" max="16384" width="8.8359375" style="11"/>
+    <col min="19" max="19" width="36.875" style="3" customWidth="1"/>
+    <col min="20" max="20" width="67.3359375" style="10" customWidth="1"/>
+    <col min="21" max="16384" width="8.8359375" style="9"/>
   </cols>
   <sheetData>
-    <row r="1" s="8" customFormat="1" spans="1:21">
+    <row r="1" s="8" customFormat="1" spans="1:20">
       <c r="A1" s="4" t="s">
         <v>0</v>
       </c>
@@ -1327,52 +1326,49 @@
       <c r="T1" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="U1" s="4" t="s">
+    </row>
+    <row r="2" s="9" customFormat="1" spans="1:20">
+      <c r="A2" s="5" t="s">
         <v>20</v>
       </c>
-    </row>
-    <row r="2" s="9" customFormat="1" spans="1:21">
-      <c r="A2" s="5" t="s">
+      <c r="B2" s="5" t="s">
         <v>21</v>
       </c>
-      <c r="B2" s="5" t="s">
+      <c r="C2" s="5">
+        <v>1</v>
+      </c>
+      <c r="D2" s="5" t="s">
         <v>22</v>
       </c>
-      <c r="C2" s="5">
-        <v>1</v>
-      </c>
-      <c r="D2" s="5" t="s">
+      <c r="E2" s="5" t="s">
         <v>23</v>
       </c>
-      <c r="E2" s="5" t="s">
+      <c r="F2" s="5">
+        <v>1</v>
+      </c>
+      <c r="G2" s="5" t="s">
         <v>24</v>
       </c>
-      <c r="F2" s="5">
-        <v>1</v>
-      </c>
-      <c r="G2" s="5" t="s">
+      <c r="H2" s="5" t="s">
         <v>25</v>
-      </c>
-      <c r="H2" s="5" t="s">
-        <v>26</v>
       </c>
       <c r="I2" s="5">
         <v>1.28</v>
       </c>
       <c r="J2" s="5" t="s">
+        <v>26</v>
+      </c>
+      <c r="K2" s="5" t="s">
         <v>27</v>
-      </c>
-      <c r="K2" s="5" t="s">
-        <v>28</v>
       </c>
       <c r="L2" s="5">
         <v>2</v>
       </c>
       <c r="M2" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="N2" s="5" t="s">
         <v>29</v>
-      </c>
-      <c r="N2" s="5" t="s">
-        <v>30</v>
       </c>
       <c r="O2" s="5">
         <v>0.5</v>
@@ -1387,57 +1383,54 @@
         <v>88</v>
       </c>
       <c r="S2" s="5">
-        <v>89.2619038609871</v>
-      </c>
-      <c r="T2" s="6">
-        <v>74.5386270183539</v>
-      </c>
-      <c r="U2" s="12" t="s">
+        <v>74.81824</v>
+      </c>
+      <c r="T2" s="11" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="3" s="9" customFormat="1" spans="1:20">
+      <c r="A3" s="5" t="s">
         <v>31</v>
       </c>
-    </row>
-    <row r="3" s="9" customFormat="1" spans="1:21">
-      <c r="A3" s="5" t="s">
+      <c r="B3" s="5" t="s">
         <v>32</v>
       </c>
-      <c r="B3" s="5" t="s">
+      <c r="C3" s="5">
+        <v>1</v>
+      </c>
+      <c r="D3" s="5" t="s">
         <v>33</v>
       </c>
-      <c r="C3" s="5">
-        <v>1</v>
-      </c>
-      <c r="D3" s="5" t="s">
+      <c r="E3" s="5" t="s">
         <v>34</v>
       </c>
-      <c r="E3" s="5" t="s">
-        <v>35</v>
-      </c>
       <c r="F3" s="5">
         <v>1</v>
       </c>
       <c r="G3" s="5" t="s">
+        <v>24</v>
+      </c>
+      <c r="H3" s="5" t="s">
         <v>25</v>
-      </c>
-      <c r="H3" s="5" t="s">
-        <v>26</v>
       </c>
       <c r="I3" s="5">
         <v>1.28</v>
       </c>
       <c r="J3" s="5" t="s">
+        <v>26</v>
+      </c>
+      <c r="K3" s="5" t="s">
         <v>27</v>
-      </c>
-      <c r="K3" s="5" t="s">
-        <v>28</v>
       </c>
       <c r="L3" s="5">
         <v>2</v>
       </c>
       <c r="M3" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="N3" s="5" t="s">
         <v>29</v>
-      </c>
-      <c r="N3" s="5" t="s">
-        <v>30</v>
       </c>
       <c r="O3" s="5">
         <v>0.5</v>
@@ -1452,57 +1445,54 @@
         <v>65</v>
       </c>
       <c r="S3" s="5">
-        <v>74.567145182145</v>
-      </c>
-      <c r="T3" s="7">
-        <v>75.6161113032893</v>
-      </c>
-      <c r="U3" s="12" t="s">
-        <v>31</v>
+        <v>70.71656</v>
+      </c>
+      <c r="T3" s="11" t="s">
+        <v>30</v>
       </c>
     </row>
-    <row r="4" s="9" customFormat="1" spans="1:21">
+    <row r="4" s="9" customFormat="1" spans="1:20">
       <c r="A4" s="5" t="s">
+        <v>35</v>
+      </c>
+      <c r="B4" s="5" t="s">
         <v>36</v>
       </c>
-      <c r="B4" s="5" t="s">
+      <c r="C4" s="5">
+        <v>1</v>
+      </c>
+      <c r="D4" s="5" t="s">
         <v>37</v>
       </c>
-      <c r="C4" s="5">
-        <v>1</v>
-      </c>
-      <c r="D4" s="5" t="s">
+      <c r="E4" s="5" t="s">
         <v>38</v>
       </c>
-      <c r="E4" s="5" t="s">
-        <v>39</v>
-      </c>
       <c r="F4" s="5">
         <v>1</v>
       </c>
       <c r="G4" s="5" t="s">
+        <v>24</v>
+      </c>
+      <c r="H4" s="5" t="s">
         <v>25</v>
-      </c>
-      <c r="H4" s="5" t="s">
-        <v>26</v>
       </c>
       <c r="I4" s="5">
         <v>1.28</v>
       </c>
       <c r="J4" s="5" t="s">
+        <v>26</v>
+      </c>
+      <c r="K4" s="5" t="s">
         <v>27</v>
-      </c>
-      <c r="K4" s="5" t="s">
-        <v>28</v>
       </c>
       <c r="L4" s="5">
         <v>2</v>
       </c>
       <c r="M4" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="N4" s="5" t="s">
         <v>29</v>
-      </c>
-      <c r="N4" s="5" t="s">
-        <v>30</v>
       </c>
       <c r="O4" s="5">
         <v>0.5</v>
@@ -1517,57 +1507,54 @@
         <v>65</v>
       </c>
       <c r="S4" s="5">
-        <v>72.0339890220673</v>
-      </c>
-      <c r="T4" s="7">
-        <v>61.9587866579012</v>
-      </c>
-      <c r="U4" s="12" t="s">
-        <v>31</v>
+        <v>75.42405</v>
+      </c>
+      <c r="T4" s="11" t="s">
+        <v>30</v>
       </c>
     </row>
-    <row r="5" s="9" customFormat="1" spans="1:21">
+    <row r="5" s="9" customFormat="1" spans="1:20">
       <c r="A5" s="5" t="s">
+        <v>39</v>
+      </c>
+      <c r="B5" s="5" t="s">
         <v>40</v>
       </c>
-      <c r="B5" s="5" t="s">
+      <c r="C5" s="5">
+        <v>1</v>
+      </c>
+      <c r="D5" s="5" t="s">
         <v>41</v>
       </c>
-      <c r="C5" s="5">
-        <v>1</v>
-      </c>
-      <c r="D5" s="5" t="s">
+      <c r="E5" s="5" t="s">
         <v>42</v>
       </c>
-      <c r="E5" s="5" t="s">
-        <v>43</v>
-      </c>
       <c r="F5" s="5">
         <v>1</v>
       </c>
       <c r="G5" s="5" t="s">
+        <v>24</v>
+      </c>
+      <c r="H5" s="5" t="s">
         <v>25</v>
-      </c>
-      <c r="H5" s="5" t="s">
-        <v>26</v>
       </c>
       <c r="I5" s="5">
         <v>1.28</v>
       </c>
       <c r="J5" s="5" t="s">
+        <v>26</v>
+      </c>
+      <c r="K5" s="5" t="s">
         <v>27</v>
-      </c>
-      <c r="K5" s="5" t="s">
-        <v>28</v>
       </c>
       <c r="L5" s="5">
         <v>2</v>
       </c>
       <c r="M5" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="N5" s="5" t="s">
         <v>29</v>
-      </c>
-      <c r="N5" s="5" t="s">
-        <v>30</v>
       </c>
       <c r="O5" s="5">
         <v>0.5</v>
@@ -1582,57 +1569,54 @@
         <v>78</v>
       </c>
       <c r="S5" s="5">
-        <v>73.0615062979917</v>
-      </c>
-      <c r="T5" s="7">
-        <v>73.2981687791631</v>
-      </c>
-      <c r="U5" s="12" t="s">
-        <v>31</v>
+        <v>60.514782</v>
+      </c>
+      <c r="T5" s="11" t="s">
+        <v>30</v>
       </c>
     </row>
-    <row r="6" s="9" customFormat="1" spans="1:21">
+    <row r="6" s="9" customFormat="1" spans="1:20">
       <c r="A6" s="5" t="s">
+        <v>43</v>
+      </c>
+      <c r="B6" s="5" t="s">
         <v>44</v>
       </c>
-      <c r="B6" s="5" t="s">
+      <c r="C6" s="5">
+        <v>1</v>
+      </c>
+      <c r="D6" s="5" t="s">
         <v>45</v>
       </c>
-      <c r="C6" s="5">
-        <v>1</v>
-      </c>
-      <c r="D6" s="5" t="s">
+      <c r="E6" s="5" t="s">
         <v>46</v>
       </c>
-      <c r="E6" s="5" t="s">
-        <v>47</v>
-      </c>
       <c r="F6" s="5">
         <v>1</v>
       </c>
       <c r="G6" s="5" t="s">
+        <v>24</v>
+      </c>
+      <c r="H6" s="5" t="s">
         <v>25</v>
-      </c>
-      <c r="H6" s="5" t="s">
-        <v>26</v>
       </c>
       <c r="I6" s="5">
         <v>1.28</v>
       </c>
       <c r="J6" s="5" t="s">
+        <v>26</v>
+      </c>
+      <c r="K6" s="5" t="s">
         <v>27</v>
-      </c>
-      <c r="K6" s="5" t="s">
-        <v>28</v>
       </c>
       <c r="L6" s="5">
         <v>2</v>
       </c>
       <c r="M6" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="N6" s="5" t="s">
         <v>29</v>
-      </c>
-      <c r="N6" s="5" t="s">
-        <v>30</v>
       </c>
       <c r="O6" s="5">
         <v>0.5</v>
@@ -1647,57 +1631,54 @@
         <v>82</v>
       </c>
       <c r="S6" s="5">
-        <v>73.1542310016332</v>
-      </c>
-      <c r="T6" s="7">
-        <v>80.6320553217847</v>
-      </c>
-      <c r="U6" s="12" t="s">
-        <v>31</v>
+        <v>58.30306</v>
+      </c>
+      <c r="T6" s="11" t="s">
+        <v>30</v>
       </c>
     </row>
-    <row r="7" s="9" customFormat="1" spans="1:21">
+    <row r="7" s="9" customFormat="1" spans="1:20">
       <c r="A7" s="5" t="s">
+        <v>47</v>
+      </c>
+      <c r="B7" s="5" t="s">
         <v>48</v>
       </c>
-      <c r="B7" s="5" t="s">
+      <c r="C7" s="5">
+        <v>1</v>
+      </c>
+      <c r="D7" s="5" t="s">
         <v>49</v>
       </c>
-      <c r="C7" s="5">
-        <v>1</v>
-      </c>
-      <c r="D7" s="5" t="s">
+      <c r="E7" s="5" t="s">
         <v>50</v>
       </c>
-      <c r="E7" s="5" t="s">
-        <v>51</v>
-      </c>
       <c r="F7" s="5">
         <v>1</v>
       </c>
       <c r="G7" s="5" t="s">
+        <v>24</v>
+      </c>
+      <c r="H7" s="5" t="s">
         <v>25</v>
-      </c>
-      <c r="H7" s="5" t="s">
-        <v>26</v>
       </c>
       <c r="I7" s="5">
         <v>1.28</v>
       </c>
       <c r="J7" s="5" t="s">
+        <v>26</v>
+      </c>
+      <c r="K7" s="5" t="s">
         <v>27</v>
-      </c>
-      <c r="K7" s="5" t="s">
-        <v>28</v>
       </c>
       <c r="L7" s="5">
         <v>2</v>
       </c>
       <c r="M7" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="N7" s="5" t="s">
         <v>29</v>
-      </c>
-      <c r="N7" s="5" t="s">
-        <v>30</v>
       </c>
       <c r="O7" s="5">
         <v>0.5</v>
@@ -1712,13 +1693,10 @@
         <v>70</v>
       </c>
       <c r="S7" s="5">
-        <v>73.1173267481458</v>
-      </c>
-      <c r="T7" s="7">
-        <v>67.137463280879</v>
-      </c>
-      <c r="U7" s="12" t="s">
-        <v>31</v>
+        <v>63.162655</v>
+      </c>
+      <c r="T7" s="11" t="s">
+        <v>30</v>
       </c>
     </row>
   </sheetData>
@@ -1810,60 +1788,60 @@
         <v>16</v>
       </c>
       <c r="R1" s="4" t="s">
+        <v>51</v>
+      </c>
+      <c r="S1" s="4" t="s">
         <v>52</v>
       </c>
-      <c r="S1" s="4" t="s">
-        <v>18</v>
-      </c>
       <c r="T1" s="4" t="s">
+        <v>53</v>
+      </c>
+      <c r="U1" s="4" t="s">
         <v>19</v>
-      </c>
-      <c r="U1" s="4" t="s">
-        <v>20</v>
       </c>
     </row>
     <row r="2" s="2" customFormat="1" spans="1:21">
       <c r="A2" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="B2" s="5" t="s">
         <v>21</v>
       </c>
-      <c r="B2" s="5" t="s">
+      <c r="C2" s="5">
+        <v>1</v>
+      </c>
+      <c r="D2" s="5" t="s">
         <v>22</v>
       </c>
-      <c r="C2" s="5">
-        <v>1</v>
-      </c>
-      <c r="D2" s="5" t="s">
+      <c r="E2" s="5" t="s">
         <v>23</v>
       </c>
-      <c r="E2" s="5" t="s">
+      <c r="F2" s="5">
+        <v>1</v>
+      </c>
+      <c r="G2" s="5" t="s">
         <v>24</v>
       </c>
-      <c r="F2" s="5">
-        <v>1</v>
-      </c>
-      <c r="G2" s="5" t="s">
+      <c r="H2" s="5" t="s">
         <v>25</v>
-      </c>
-      <c r="H2" s="5" t="s">
-        <v>26</v>
       </c>
       <c r="I2" s="5">
         <v>1.28</v>
       </c>
       <c r="J2" s="5" t="s">
+        <v>26</v>
+      </c>
+      <c r="K2" s="5" t="s">
         <v>27</v>
-      </c>
-      <c r="K2" s="5" t="s">
-        <v>28</v>
       </c>
       <c r="L2" s="5">
         <v>2</v>
       </c>
       <c r="M2" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="N2" s="5" t="s">
         <v>29</v>
-      </c>
-      <c r="N2" s="5" t="s">
-        <v>30</v>
       </c>
       <c r="O2" s="5">
         <v>0.5</v>
@@ -1884,51 +1862,51 @@
         <v>74.5386270183539</v>
       </c>
       <c r="U2" s="5" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
     </row>
     <row r="3" s="2" customFormat="1" spans="1:21">
       <c r="A3" s="5" t="s">
+        <v>31</v>
+      </c>
+      <c r="B3" s="5" t="s">
         <v>32</v>
       </c>
-      <c r="B3" s="5" t="s">
+      <c r="C3" s="5">
+        <v>1</v>
+      </c>
+      <c r="D3" s="5" t="s">
         <v>33</v>
       </c>
-      <c r="C3" s="5">
-        <v>1</v>
-      </c>
-      <c r="D3" s="5" t="s">
+      <c r="E3" s="5" t="s">
         <v>34</v>
       </c>
-      <c r="E3" s="5" t="s">
-        <v>35</v>
-      </c>
       <c r="F3" s="5">
         <v>1</v>
       </c>
       <c r="G3" s="5" t="s">
+        <v>24</v>
+      </c>
+      <c r="H3" s="5" t="s">
         <v>25</v>
-      </c>
-      <c r="H3" s="5" t="s">
-        <v>26</v>
       </c>
       <c r="I3" s="5">
         <v>1.28</v>
       </c>
       <c r="J3" s="5" t="s">
+        <v>26</v>
+      </c>
+      <c r="K3" s="5" t="s">
         <v>27</v>
-      </c>
-      <c r="K3" s="5" t="s">
-        <v>28</v>
       </c>
       <c r="L3" s="5">
         <v>2</v>
       </c>
       <c r="M3" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="N3" s="5" t="s">
         <v>29</v>
-      </c>
-      <c r="N3" s="5" t="s">
-        <v>30</v>
       </c>
       <c r="O3" s="5">
         <v>0.5</v>
@@ -1949,51 +1927,51 @@
         <v>75.6161113032893</v>
       </c>
       <c r="U3" s="5" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
     </row>
     <row r="4" s="2" customFormat="1" spans="1:21">
       <c r="A4" s="5" t="s">
+        <v>35</v>
+      </c>
+      <c r="B4" s="5" t="s">
         <v>36</v>
       </c>
-      <c r="B4" s="5" t="s">
+      <c r="C4" s="5">
+        <v>1</v>
+      </c>
+      <c r="D4" s="5" t="s">
         <v>37</v>
       </c>
-      <c r="C4" s="5">
-        <v>1</v>
-      </c>
-      <c r="D4" s="5" t="s">
+      <c r="E4" s="5" t="s">
         <v>38</v>
       </c>
-      <c r="E4" s="5" t="s">
-        <v>39</v>
-      </c>
       <c r="F4" s="5">
         <v>1</v>
       </c>
       <c r="G4" s="5" t="s">
+        <v>24</v>
+      </c>
+      <c r="H4" s="5" t="s">
         <v>25</v>
-      </c>
-      <c r="H4" s="5" t="s">
-        <v>26</v>
       </c>
       <c r="I4" s="5">
         <v>1.28</v>
       </c>
       <c r="J4" s="5" t="s">
+        <v>26</v>
+      </c>
+      <c r="K4" s="5" t="s">
         <v>27</v>
-      </c>
-      <c r="K4" s="5" t="s">
-        <v>28</v>
       </c>
       <c r="L4" s="5">
         <v>2</v>
       </c>
       <c r="M4" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="N4" s="5" t="s">
         <v>29</v>
-      </c>
-      <c r="N4" s="5" t="s">
-        <v>30</v>
       </c>
       <c r="O4" s="5">
         <v>0.5</v>
@@ -2014,51 +1992,51 @@
         <v>61.9587866579012</v>
       </c>
       <c r="U4" s="5" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
     </row>
     <row r="5" s="2" customFormat="1" spans="1:21">
       <c r="A5" s="5" t="s">
+        <v>39</v>
+      </c>
+      <c r="B5" s="5" t="s">
         <v>40</v>
       </c>
-      <c r="B5" s="5" t="s">
+      <c r="C5" s="5">
+        <v>1</v>
+      </c>
+      <c r="D5" s="5" t="s">
         <v>41</v>
       </c>
-      <c r="C5" s="5">
-        <v>1</v>
-      </c>
-      <c r="D5" s="5" t="s">
+      <c r="E5" s="5" t="s">
         <v>42</v>
       </c>
-      <c r="E5" s="5" t="s">
-        <v>43</v>
-      </c>
       <c r="F5" s="5">
         <v>1</v>
       </c>
       <c r="G5" s="5" t="s">
+        <v>24</v>
+      </c>
+      <c r="H5" s="5" t="s">
         <v>25</v>
-      </c>
-      <c r="H5" s="5" t="s">
-        <v>26</v>
       </c>
       <c r="I5" s="5">
         <v>1.28</v>
       </c>
       <c r="J5" s="5" t="s">
+        <v>26</v>
+      </c>
+      <c r="K5" s="5" t="s">
         <v>27</v>
-      </c>
-      <c r="K5" s="5" t="s">
-        <v>28</v>
       </c>
       <c r="L5" s="5">
         <v>2</v>
       </c>
       <c r="M5" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="N5" s="5" t="s">
         <v>29</v>
-      </c>
-      <c r="N5" s="5" t="s">
-        <v>30</v>
       </c>
       <c r="O5" s="5">
         <v>0.5</v>
@@ -2079,51 +2057,51 @@
         <v>73.2981687791631</v>
       </c>
       <c r="U5" s="5" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
     </row>
     <row r="6" s="2" customFormat="1" spans="1:21">
       <c r="A6" s="5" t="s">
+        <v>43</v>
+      </c>
+      <c r="B6" s="5" t="s">
         <v>44</v>
       </c>
-      <c r="B6" s="5" t="s">
+      <c r="C6" s="5">
+        <v>1</v>
+      </c>
+      <c r="D6" s="5" t="s">
         <v>45</v>
       </c>
-      <c r="C6" s="5">
-        <v>1</v>
-      </c>
-      <c r="D6" s="5" t="s">
+      <c r="E6" s="5" t="s">
         <v>46</v>
       </c>
-      <c r="E6" s="5" t="s">
-        <v>47</v>
-      </c>
       <c r="F6" s="5">
         <v>1</v>
       </c>
       <c r="G6" s="5" t="s">
+        <v>24</v>
+      </c>
+      <c r="H6" s="5" t="s">
         <v>25</v>
-      </c>
-      <c r="H6" s="5" t="s">
-        <v>26</v>
       </c>
       <c r="I6" s="5">
         <v>1.28</v>
       </c>
       <c r="J6" s="5" t="s">
+        <v>26</v>
+      </c>
+      <c r="K6" s="5" t="s">
         <v>27</v>
-      </c>
-      <c r="K6" s="5" t="s">
-        <v>28</v>
       </c>
       <c r="L6" s="5">
         <v>2</v>
       </c>
       <c r="M6" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="N6" s="5" t="s">
         <v>29</v>
-      </c>
-      <c r="N6" s="5" t="s">
-        <v>30</v>
       </c>
       <c r="O6" s="5">
         <v>0.5</v>
@@ -2144,51 +2122,51 @@
         <v>80.6320553217847</v>
       </c>
       <c r="U6" s="5" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
     </row>
     <row r="7" s="2" customFormat="1" spans="1:21">
       <c r="A7" s="5" t="s">
+        <v>47</v>
+      </c>
+      <c r="B7" s="5" t="s">
         <v>48</v>
       </c>
-      <c r="B7" s="5" t="s">
+      <c r="C7" s="5">
+        <v>1</v>
+      </c>
+      <c r="D7" s="5" t="s">
         <v>49</v>
       </c>
-      <c r="C7" s="5">
-        <v>1</v>
-      </c>
-      <c r="D7" s="5" t="s">
+      <c r="E7" s="5" t="s">
         <v>50</v>
       </c>
-      <c r="E7" s="5" t="s">
-        <v>51</v>
-      </c>
       <c r="F7" s="5">
         <v>1</v>
       </c>
       <c r="G7" s="5" t="s">
+        <v>24</v>
+      </c>
+      <c r="H7" s="5" t="s">
         <v>25</v>
-      </c>
-      <c r="H7" s="5" t="s">
-        <v>26</v>
       </c>
       <c r="I7" s="5">
         <v>1.28</v>
       </c>
       <c r="J7" s="5" t="s">
+        <v>26</v>
+      </c>
+      <c r="K7" s="5" t="s">
         <v>27</v>
-      </c>
-      <c r="K7" s="5" t="s">
-        <v>28</v>
       </c>
       <c r="L7" s="5">
         <v>2</v>
       </c>
       <c r="M7" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="N7" s="5" t="s">
         <v>29</v>
-      </c>
-      <c r="N7" s="5" t="s">
-        <v>30</v>
       </c>
       <c r="O7" s="5">
         <v>0.5</v>
@@ -2209,7 +2187,7 @@
         <v>67.137463280879</v>
       </c>
       <c r="U7" s="5" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
     </row>
   </sheetData>

</xml_diff>